<commit_message>
scan: seg5 2026-08-17 17:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-08-17.xlsx
+++ b/output/full_scan/batch_seq6_2026-08-17.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O113"/>
+  <dimension ref="A1:O114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2170,21 +2170,21 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6291</v>
+        <v>6217</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>中探針</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>511.3716087262496</v>
+        <v>512.7931349871168</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>393.5</v>
+        <v>171</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>49.31901558250722</v>
+        <v>49.63493895378722</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22.17769134685688</v>
+        <v>19.80147032479681</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.7793675093060006</v>
+        <v>0.2302482817141759</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,51 +2213,51 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>10.92367545177764</v>
+        <v>7.683302607387244</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6218</v>
+        <v>6291</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>509.1155304340584</v>
+        <v>511.3716087262496</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>35.6</v>
+        <v>393.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G34" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.13817943422897</v>
+        <v>49.31901558250722</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>14.32309149578834</v>
+        <v>22.17769134685688</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.91566730118506</v>
+        <v>0.7793675093060006</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.4900538371533342</v>
+        <v>10.92367545177764</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6175</v>
+        <v>6218</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>504.09381497429</v>
+        <v>509.1155304340584</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>77.40000000000001</v>
+        <v>35.6</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>42.16041135552752</v>
+        <v>54.13817943422897</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>21.5579104480765</v>
+        <v>14.32309149578834</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.7795460444498482</v>
+        <v>0.91566730118506</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>1.142028495252714</v>
+        <v>0.4900538371533342</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6223</v>
+        <v>6175</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>476.4049677826968</v>
+        <v>504.09381497429</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>6440</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,49 +2354,49 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>55.75487750802456</v>
+        <v>42.16041135552752</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>16.51037729568007</v>
+        <v>21.5579104480765</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.5898786219119773</v>
+        <v>0.7795460444498482</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>113.2136490688242</v>
+        <v>1.142028495252714</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6207</v>
+        <v>6223</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>雷科</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>476.2227126265672</v>
+        <v>476.4049677826968</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>107.5</v>
+        <v>6440</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,69 +2407,69 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>45.80030262072125</v>
+        <v>55.75487750802456</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>19.12176378687617</v>
+        <v>16.51037729568007</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.6188100399583727</v>
+        <v>0.5898786219119773</v>
       </c>
       <c r="K37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L37" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M37" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1.741082202864016</v>
+        <v>113.2136490688242</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6191</v>
+        <v>6207</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>雷科</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>456.3707363795792</v>
+        <v>476.2227126265672</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>85.8</v>
+        <v>107.5</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G38" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>43.99379742200224</v>
+        <v>45.80030262072125</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>28.14776711011619</v>
+        <v>19.12176378687617</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.5171908721713937</v>
+        <v>0.6188100399583727</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.8117038289605016</v>
+        <v>1.741082202864016</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6192</v>
+        <v>6191</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>453.7115874211973</v>
+        <v>456.3707363795792</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>117</v>
+        <v>85.8</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>50.94037961170752</v>
+        <v>43.99379742200224</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>21.65150125594516</v>
+        <v>28.14776711011619</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.5097021011355406</v>
+        <v>0.5171908721713937</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.7682016232961034</v>
+        <v>0.8117038289605016</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6271</v>
+        <v>6192</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>449.5762420948677</v>
+        <v>453.7115874211973</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>198</v>
+        <v>117</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>49.62177635141473</v>
+        <v>50.94037961170752</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>17.90248563691822</v>
+        <v>21.65150125594516</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.4303276635932443</v>
+        <v>0.5097021011355406</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>4.307352043953145</v>
+        <v>0.7682016232961034</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6202</v>
+        <v>6271</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>盛群</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>445.1726287642916</v>
+        <v>449.5762420948677</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>60.3</v>
+        <v>198</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>50.62311902646113</v>
+        <v>49.62177635141473</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>15.88317915155272</v>
+        <v>17.90248563691822</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.3363590921591714</v>
+        <v>0.4303276635932443</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.7581711556892641</v>
+        <v>4.307352043953145</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2647,21 +2647,21 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6290</v>
+        <v>6202</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>良維</t>
+          <t>盛群</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>436.3192509973358</v>
+        <v>445.1726287642916</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>216</v>
+        <v>60.3</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>40.30838265440747</v>
+        <v>50.62311902646113</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>33.82465057255358</v>
+        <v>15.88317915155272</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.607145361524434</v>
+        <v>0.3363590921591714</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,51 +2690,51 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>3.5566656064791</v>
+        <v>0.7581711556892641</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6288</v>
+        <v>6290</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>聯嘉</t>
+          <t>良維</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>435.5265223214369</v>
+        <v>436.3192509973358</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>20.95</v>
+        <v>216</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2025-08-04</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G43" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>58.74221727490784</v>
+        <v>40.30838265440747</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>26.73403069733332</v>
+        <v>33.82465057255358</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.6831032524092705</v>
+        <v>0.607145361524434</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,51 +2743,51 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0005753878569035</v>
+        <v>3.5566656064791</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6415</v>
+        <v>6288</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>聯嘉</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>432.4816746745823</v>
+        <v>435.5265223214369</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>453.5</v>
+        <v>20.95</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2025-08-04</t>
         </is>
       </c>
       <c r="G44" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>47.1877596455715</v>
+        <v>58.74221727490784</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>15.58670752635502</v>
+        <v>26.73403069733332</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.7743070033943384</v>
+        <v>0.6831032524092705</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,48 +2796,48 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>8.601860666240061</v>
+        <v>0.0005753878569035</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6188</v>
+        <v>6415</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>432.2578091449213</v>
+        <v>432.4816746745823</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>453.5</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G45" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>45.19644952818049</v>
+        <v>47.1877596455715</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>20.79335693109767</v>
+        <v>15.58670752635502</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.5451483402180791</v>
+        <v>0.7743070033943384</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,48 +2849,48 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.67008217700196</v>
+        <v>8.601860666240061</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6196</v>
+        <v>6188</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>廣明</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>428.3695624691297</v>
+        <v>432.2578091449213</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>511</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G46" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>50.14224349324682</v>
+        <v>45.19644952818049</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>13.24842390275525</v>
+        <v>20.79335693109767</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.7058900062634257</v>
+        <v>0.5451483402180791</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>2.921544777679355</v>
+        <v>0.67008217700196</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6405</v>
+        <v>6196</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>悅城</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>424.9936674716879</v>
+        <v>428.3695624691297</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>39.65</v>
+        <v>511</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>40.16851676606112</v>
+        <v>50.14224349324682</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>27.39025700501334</v>
+        <v>13.24842390275525</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.406455108979947</v>
+        <v>0.7058900062634257</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>1.210556868633968</v>
+        <v>2.921544777679355</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6261</v>
+        <v>6405</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>悅城</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>424.7780478644028</v>
+        <v>424.9936674716879</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>77.8</v>
+        <v>39.65</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>40.11191102596668</v>
+        <v>40.16851676606112</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>31.59322447207921</v>
+        <v>27.39025700501334</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.4059776950350834</v>
+        <v>0.406455108979947</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.8607990556058667</v>
+        <v>1.210556868633968</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3018,21 +3018,21 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6284</v>
+        <v>6261</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>佳邦</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>422.6959584933393</v>
+        <v>424.7780478644028</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>77.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>45.02888683715207</v>
+        <v>40.11191102596668</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.6420753335839</v>
+        <v>31.59322447207921</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.5200581825100142</v>
+        <v>0.4059776950350834</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>1.296660118973392</v>
+        <v>0.8607990556058667</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6230</v>
+        <v>6284</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>佳邦</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>422.4883907782477</v>
+        <v>422.6959584933393</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>112</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>46.96460163125898</v>
+        <v>45.02888683715207</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>24.67462519328448</v>
+        <v>23.6420753335839</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.5568522572882527</v>
+        <v>0.5200581825100142</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.8888857763924252</v>
+        <v>1.296660118973392</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6274</v>
+        <v>6230</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>422.1458328528701</v>
+        <v>422.4883907782477</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1600</v>
+        <v>112</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>58.08017171976171</v>
+        <v>46.96460163125898</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>14.39462268238496</v>
+        <v>24.67462519328448</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.162611434984773</v>
+        <v>0.5568522572882527</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,48 +3167,48 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>49.72899119019309</v>
+        <v>0.8888857763924252</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6227</v>
+        <v>6274</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>茂綸</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>421.0908510361546</v>
+        <v>422.1458328528701</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>124</v>
+        <v>1600</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G52" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>54.77799736907603</v>
+        <v>58.08017171976171</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>16.30442663557631</v>
+        <v>14.39462268238496</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.7986527453172103</v>
+        <v>1.162611434984773</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,48 +3220,48 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1.198271256388733</v>
+        <v>49.72899119019309</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6257</v>
+        <v>6227</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>419.9646125557714</v>
+        <v>421.0908510361546</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>208</v>
+        <v>124</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G53" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.53282945674135</v>
+        <v>54.77799736907603</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>15.27630563787065</v>
+        <v>16.30442663557631</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.5186615743219362</v>
+        <v>0.7986527453172103</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>2.058137627934711</v>
+        <v>1.198271256388733</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3283,21 +3283,21 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6416</v>
+        <v>6257</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>419.3647678367519</v>
+        <v>419.9646125557714</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>95.09999999999999</v>
+        <v>208</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>49.00566401230763</v>
+        <v>48.53282945674135</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>17.96591333845268</v>
+        <v>15.27630563787065</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.2418575236600208</v>
+        <v>0.5186615743219362</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.6948951367677765</v>
+        <v>2.058137627934711</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6263</v>
+        <v>6416</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>普萊德</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>414.9765115595573</v>
+        <v>419.3647678367519</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>163</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>56.84952475939082</v>
+        <v>49.00566401230763</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>10.83947284594204</v>
+        <v>17.96591333845268</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.5449019306280675</v>
+        <v>0.2418575236600208</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.881436997211398</v>
+        <v>-0.6948951367677765</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6442</v>
+        <v>6263</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>普萊德</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>410.3103149225057</v>
+        <v>414.9765115595573</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>1630</v>
+        <v>163</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>59.81887008947148</v>
+        <v>56.84952475939082</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>20.34752138450064</v>
+        <v>10.83947284594204</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.05567346059406</v>
+        <v>0.5449019306280675</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>55.25455742820381</v>
+        <v>1.881436997211398</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6197</v>
+        <v>6442</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>佳必琪</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>409.7390158132921</v>
+        <v>410.3103149225057</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>301.5</v>
+        <v>1630</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.78922379913223</v>
+        <v>59.81887008947148</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>15.79054625264239</v>
+        <v>20.34752138450064</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.3740451197781749</v>
+        <v>1.05567346059406</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.373334888374628</v>
+        <v>55.25455742820381</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6443</v>
+        <v>6197</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>元晶</t>
+          <t>佳必琪</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>406.9226960413878</v>
+        <v>409.7390158132921</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>28.05</v>
+        <v>301.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>48.8380783445638</v>
+        <v>46.78922379913223</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>21.96245378626197</v>
+        <v>15.79054625264239</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.052404359463636</v>
+        <v>0.3740451197781749</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,48 +3538,48 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.6215442953112675</v>
+        <v>1.373334888374628</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6241</v>
+        <v>6443</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>鑫永洋</t>
+          <t>元晶</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>404.2112111417101</v>
+        <v>406.9226960413878</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>13.8</v>
+        <v>28.05</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G59" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>37.42739215537994</v>
+        <v>48.8380783445638</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>23.28506702190436</v>
+        <v>21.96245378626197</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.9016594149431636</v>
+        <v>1.052404359463636</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,48 +3591,48 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.3702590279394657</v>
+        <v>0.6215442953112675</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6464</v>
+        <v>6241</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>台數科</t>
+          <t>鑫永洋</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>403.1650936235583</v>
+        <v>404.2112111417101</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>78</v>
+        <v>13.8</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G60" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>49.6842122698114</v>
+        <v>37.42739215537994</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>28.22290506986554</v>
+        <v>23.28506702190436</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.3771627717807023</v>
+        <v>0.9016594149431636</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0909648165073899</v>
+        <v>-0.3702590279394657</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6418</v>
+        <v>6464</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>詠昇</t>
+          <t>台數科</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>392.2909071965701</v>
+        <v>403.1650936235583</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>32.15</v>
+        <v>78</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>52.83826577212653</v>
+        <v>49.6842122698114</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>17.64457690471677</v>
+        <v>28.22290506986554</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.5160161151161801</v>
+        <v>0.3771627717807023</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,51 +3697,51 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1093795771153092</v>
+        <v>-0.0909648165073899</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6198</v>
+        <v>6418</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>詠昇</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>387.4845954139302</v>
+        <v>392.2909071965701</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>19.8</v>
+        <v>32.15</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G62" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>51.80677993877924</v>
+        <v>52.83826577212653</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>7.517367369667177</v>
+        <v>17.64457690471677</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2.548459541393023</v>
+        <v>0.5160161151161801</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,51 +3750,51 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.9631492879062996</v>
+        <v>0.1093795771153092</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6462</v>
+        <v>6198</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>神盾</t>
+          <t>瑞築</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>383.7087145786928</v>
+        <v>387.4845954139302</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>99.7</v>
+        <v>19.8</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G63" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.99224225219311</v>
+        <v>51.80677993877924</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>16.5596648231879</v>
+        <v>7.517367369667177</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.5706398164424321</v>
+        <v>2.548459541393023</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.140336750209126</v>
+        <v>0.9631492879062996</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6168</v>
+        <v>6462</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>宏齊</t>
+          <t>神盾</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>381.216913839617</v>
+        <v>383.7087145786928</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>24.75</v>
+        <v>99.7</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>48.95740609920828</v>
+        <v>45.99224225219311</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.06429967866282</v>
+        <v>16.5596648231879</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.4340307519046507</v>
+        <v>0.5706398164424321</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,48 +3856,48 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.35967827913934</v>
+        <v>1.140336750209126</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6190</v>
+        <v>6168</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>宏齊</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>372.1543449378186</v>
+        <v>381.216913839617</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>67</v>
+        <v>24.75</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G65" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>43.91889553270983</v>
+        <v>48.95740609920828</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>29.30731838542146</v>
+        <v>16.06429967866282</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.794634932982938</v>
+        <v>0.4340307519046507</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,48 +3909,48 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.7368775660268265</v>
+        <v>0.35967827913934</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6417</v>
+        <v>6190</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>韋僑</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>368.8419745509891</v>
+        <v>372.1543449378186</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G66" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>40.02773116417124</v>
+        <v>43.91889553270983</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>23.85291944219667</v>
+        <v>29.30731838542146</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.64827156338432</v>
+        <v>0.794634932982938</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.1360690929354029</v>
+        <v>0.7368775660268265</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6165</v>
+        <v>6417</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>韋僑</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>362.0222010873141</v>
+        <v>368.8419745509891</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>47.6</v>
+        <v>110</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>41.45515301917718</v>
+        <v>40.02773116417124</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>12.82477543079827</v>
+        <v>23.85291944219667</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.618336684416959</v>
+        <v>0.64827156338432</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,51 +4015,51 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.1367452757201033</v>
+        <v>0.1360690929354029</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6237</v>
+        <v>6165</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>359.6958785503525</v>
+        <v>362.0222010873141</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>34.1</v>
+        <v>47.6</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G68" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>41.54927594809547</v>
+        <v>41.45515301917718</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>29.83907255781459</v>
+        <v>12.82477543079827</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.5416638027729617</v>
+        <v>0.618336684416959</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,51 +4068,51 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.5803439838742581</v>
+        <v>-0.1367452757201033</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6409</v>
+        <v>6237</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>旭隼</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>357.7039467357801</v>
+        <v>359.6958785503525</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>983</v>
+        <v>34.1</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G69" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>48.99815799014666</v>
+        <v>41.54927594809547</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.89471143165664</v>
+        <v>29.83907255781459</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.7666115210400173</v>
+        <v>0.5416638027729617</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,48 +4121,48 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>1.684398684027378</v>
+        <v>0.5803439838742581</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6176</v>
+        <v>6409</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>旭隼</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>357.6513352023769</v>
+        <v>357.7039467357801</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>81.3</v>
+        <v>983</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G70" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>36.44665883253602</v>
+        <v>48.99815799014666</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.2046564567175</v>
+        <v>15.89471143165664</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1.005858288434822</v>
+        <v>0.7666115210400173</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,48 +4174,48 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.1723411053592181</v>
+        <v>1.684398684027378</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6456</v>
+        <v>6176</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>356.8756533495047</v>
+        <v>357.6513352023769</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>66.5</v>
+        <v>81.3</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G71" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>52.74662258728933</v>
+        <v>36.44665883253602</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>17.0956868082101</v>
+        <v>23.2046564567175</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4693088826803875</v>
+        <v>1.005858288434822</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>1.248819506644412</v>
+        <v>-0.1723411053592181</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6432</v>
+        <v>6456</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>今展科</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>350.3655293891704</v>
+        <v>356.8756533495047</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>71.5</v>
+        <v>66.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.4758004172251</v>
+        <v>52.74662258728933</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>11.30019406203374</v>
+        <v>17.0956868082101</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.2755694728230103</v>
+        <v>0.4693088826803875</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.005826504233612</v>
+        <v>1.248819506644412</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6166</v>
+        <v>6432</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>凌華</t>
+          <t>今展科</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>350.1832550496408</v>
+        <v>350.3655293891704</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>128</v>
+        <v>71.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>45.42287694047219</v>
+        <v>48.4758004172251</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>13.43703787964442</v>
+        <v>11.30019406203374</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.4523416622165732</v>
+        <v>0.2755694728230103</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.8557831670660577</v>
+        <v>-0.005826504233612</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6209</v>
+        <v>6166</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>凌華</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>348.8280976751978</v>
+        <v>350.1832550496408</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>71.09999999999999</v>
+        <v>128</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>47.98264483672435</v>
+        <v>45.42287694047219</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>13.5389945824601</v>
+        <v>13.43703787964442</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.9908361324290454</v>
+        <v>0.4523416622165732</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.6564270773283758</v>
+        <v>-0.8557831670660577</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6275</v>
+        <v>6209</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>元山</t>
+          <t>今國光</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>345.4059452203888</v>
+        <v>348.8280976751978</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>43.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>43.38362543790127</v>
+        <v>47.98264483672435</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.13445543075047</v>
+        <v>13.5389945824601</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.4312610074231019</v>
+        <v>0.9908361324290454</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.2926292169534501</v>
+        <v>0.6564270773283758</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6243</v>
+        <v>6275</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>迅杰</t>
+          <t>元山</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>344.5290449613869</v>
+        <v>345.4059452203888</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>45.7</v>
+        <v>43.2</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>49.97231576167537</v>
+        <v>43.38362543790127</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>19.1856248324083</v>
+        <v>20.13445543075047</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.6102618188817823</v>
+        <v>0.4312610074231019</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.7737665276559091</v>
+        <v>0.2926292169534501</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6472</v>
+        <v>6243</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>保瑞</t>
+          <t>迅杰</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>343.6693854992855</v>
+        <v>344.5290449613869</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>416</v>
+        <v>45.7</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.41714401186971</v>
+        <v>49.97231576167537</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>23.82271088424895</v>
+        <v>19.1856248324083</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.5280345065006132</v>
+        <v>0.6102618188817823</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>1.729184987211692</v>
+        <v>-0.7737665276559091</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6282</v>
+        <v>6472</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>康舒</t>
+          <t>保瑞</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>343.2135870749404</v>
+        <v>343.6693854992855</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>46.55</v>
+        <v>416</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>44.41273716042204</v>
+        <v>52.41714401186971</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>17.81848053913793</v>
+        <v>23.82271088424895</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5599060491802045</v>
+        <v>0.5280345065006132</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.5813825512818673</v>
+        <v>1.729184987211692</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6441</v>
+        <v>6282</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>廣錠</t>
+          <t>康舒</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>340.5611218626414</v>
+        <v>343.2135870749404</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>22.05</v>
+        <v>46.55</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>52.97501559399221</v>
+        <v>44.41273716042204</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>21.88091927008334</v>
+        <v>17.81848053913793</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.5185206024247672</v>
+        <v>0.5599060491802045</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.3010437564805369</v>
+        <v>0.5813825512818673</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6414</v>
+        <v>6441</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>廣錠</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>333.6643711719624</v>
+        <v>340.5611218626414</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>417.5</v>
+        <v>22.05</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>46.23325917914092</v>
+        <v>52.97501559399221</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>18.58872238571707</v>
+        <v>21.88091927008334</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.4820142340799499</v>
+        <v>0.5185206024247672</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-6.549601327066707</v>
+        <v>0.3010437564805369</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6226</v>
+        <v>6414</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>光鼎</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>329.1447073140617</v>
+        <v>333.6643711719624</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>19.2</v>
+        <v>417.5</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>45.43174415578625</v>
+        <v>46.23325917914092</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.31138096747075</v>
+        <v>18.58872238571707</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.3417878042046923</v>
+        <v>0.4820142340799499</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.3670911841917343</v>
+        <v>-6.549601327066707</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6239</v>
+        <v>6226</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>318.3377812528308</v>
+        <v>329.1447073140617</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>278</v>
+        <v>19.2</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>49.55756978289645</v>
+        <v>45.43174415578625</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>13.66050366669278</v>
+        <v>16.31138096747075</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.3887568517487684</v>
+        <v>0.3417878042046923</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>4.824707137302793</v>
+        <v>-0.3670911841917343</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6164</v>
+        <v>6239</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>華興</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>310.269270758949</v>
+        <v>318.3377812528308</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>12</v>
+        <v>278</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>46.10598593406986</v>
+        <v>49.55756978289645</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>27.18631403171499</v>
+        <v>13.66050366669278</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.6197800599848817</v>
+        <v>0.3887568517487684</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0978398262911907</v>
+        <v>4.824707137302793</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6205</v>
+        <v>6164</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>詮欣</t>
+          <t>華興</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>293.19441827984</v>
+        <v>310.269270758949</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>47.48539201775861</v>
+        <v>46.10598593406986</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>22.34082821814683</v>
+        <v>27.18631403171499</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.3596814310978071</v>
+        <v>0.6197800599848817</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>1.196130511010544</v>
+        <v>0.0978398262911907</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4926,41 +4926,41 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6208</v>
+        <v>6205</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>日揚</t>
+          <t>詮欣</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>291.8199242888043</v>
+        <v>293.19441827984</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G85" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>45.07303181109776</v>
+        <v>47.48539201775861</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>13.22931155513177</v>
+        <v>22.34082821814683</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5589557006969068</v>
+        <v>0.3596814310978071</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,51 +4969,51 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.354197895591497</v>
+        <v>1.196130511010544</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6266</v>
+        <v>6208</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>泰詠</t>
+          <t>日揚</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>283.2658867283822</v>
+        <v>291.8199242888043</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>25.1</v>
+        <v>82</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G86" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>52.27710932039468</v>
+        <v>45.07303181109776</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>16.20293276998097</v>
+        <v>13.22931155513177</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.3037438766041689</v>
+        <v>0.5589557006969068</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.1685227428014753</v>
+        <v>0.354197895591497</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6270</v>
+        <v>6266</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>倍微</t>
+          <t>泰詠</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>278.0758315298505</v>
+        <v>283.2658867283822</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>30.55</v>
+        <v>25.1</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.37397841605124</v>
+        <v>52.27710932039468</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>13.9596681438122</v>
+        <v>16.20293276998097</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.3497001010762895</v>
+        <v>0.3037438766041689</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.3701409167921909</v>
+        <v>0.1685227428014753</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6272</v>
+        <v>6270</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>驊陞</t>
+          <t>倍微</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>277.9507670838748</v>
+        <v>278.0758315298505</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>23.8</v>
+        <v>30.55</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>35.19022186178162</v>
+        <v>48.37397841605124</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>41.68872831750505</v>
+        <v>13.9596681438122</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.8232828349830604</v>
+        <v>0.3497001010762895</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,48 +5128,48 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.15196433130985</v>
+        <v>0.3701409167921909</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6170</v>
+        <v>6272</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>統振</t>
+          <t>驊陞</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>277.4973202391515</v>
+        <v>277.9507670838748</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>47</v>
+        <v>23.8</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G89" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>44.59340316212784</v>
+        <v>35.19022186178162</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>32.24774964251205</v>
+        <v>41.68872831750505</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5879909560453201</v>
+        <v>0.8232828349830604</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,48 +5181,48 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.2632363192154139</v>
+        <v>0.15196433130985</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6276</v>
+        <v>6170</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>安鈦克</t>
+          <t>統振</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>263.9078411641606</v>
+        <v>277.4973202391515</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>19.15</v>
+        <v>47</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G90" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>36.65629790173665</v>
+        <v>44.59340316212784</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>28.61783326411971</v>
+        <v>32.24774964251205</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.7530872868317725</v>
+        <v>0.5879909560453201</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,51 +5234,51 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0496078529338228</v>
+        <v>0.2632363192154139</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6167</v>
+        <v>6276</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>安鈦克</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>260.690192199497</v>
+        <v>263.9078411641606</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>10.4</v>
+        <v>19.15</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G91" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>40.73075563590629</v>
+        <v>36.65629790173665</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>20.19457001355831</v>
+        <v>28.61783326411971</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.060233635570114</v>
+        <v>0.7530872868317725</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,51 +5287,51 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0540917657614959</v>
+        <v>0.0496078529338228</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6470</v>
+        <v>6167</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>宇智</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>250.9548372176272</v>
+        <v>260.690192199497</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>42.25</v>
+        <v>10.4</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G92" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>27.20122732608255</v>
+        <v>40.73075563590629</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>43.86484685355894</v>
+        <v>20.19457001355831</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4528524407372066</v>
+        <v>1.060233635570114</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0437306494325078</v>
+        <v>0.0540917657614959</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6283</v>
+        <v>6470</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>淳安</t>
+          <t>宇智</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>249.2055955620111</v>
+        <v>250.9548372176272</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>20.3</v>
+        <v>42.25</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>39.8908231072268</v>
+        <v>27.20122732608255</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>38.55674918335564</v>
+        <v>43.86484685355894</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.8340945069210504</v>
+        <v>0.4528524407372066</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.1170729196441116</v>
+        <v>-0.0437306494325078</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5403,38 +5403,38 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6220</v>
+        <v>6283</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>岳豐</t>
+          <t>淳安</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>244.4179190908388</v>
+        <v>249.2055955620111</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>25.65</v>
+        <v>20.3</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G94" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>37.0273379328901</v>
+        <v>39.8908231072268</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>29.13749832675557</v>
+        <v>38.55674918335564</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.7333861865614809</v>
+        <v>0.8340945069210504</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,48 +5446,48 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.2316773984624902</v>
+        <v>0.1170729196441116</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6201</v>
+        <v>6220</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>岳豐</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>243.0912358777546</v>
+        <v>244.4179190908388</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>45.1</v>
+        <v>25.65</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G95" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>28.90990512211095</v>
+        <v>37.0273379328901</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>19.76762430805406</v>
+        <v>29.13749832675557</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>2.135043397523185</v>
+        <v>0.7333861865614809</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,48 +5499,48 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.2674020284838551</v>
+        <v>0.2316773984624902</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6210</v>
+        <v>6201</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>慶生</t>
+          <t>亞弘電</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>240.0372865451418</v>
+        <v>243.0912358777546</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>17.75</v>
+        <v>45.1</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G96" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>50.21311050695917</v>
+        <v>28.90990512211095</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.57730933728291</v>
+        <v>19.76762430805406</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.1303700719553272</v>
+        <v>2.135043397523185</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,48 +5552,48 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.20759716625034</v>
+        <v>-0.2674020284838551</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6285</v>
+        <v>6210</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>慶生</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>238.1347109325893</v>
+        <v>240.0372865451418</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>243</v>
+        <v>17.75</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G97" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.40230189404605</v>
+        <v>50.21311050695917</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>15.9712947954258</v>
+        <v>11.57730933728291</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3718744749965058</v>
+        <v>0.1303700719553272</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>1.393517170347966</v>
+        <v>0.20759716625034</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6236</v>
+        <v>6285</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>中湛</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>232.1255164811716</v>
+        <v>238.1347109325893</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>46.8297117891449</v>
+        <v>48.40230189404605</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>9.667865126411858</v>
+        <v>15.9712947954258</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0</v>
+        <v>0.3718744749965058</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,48 +5658,48 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.4029301965684577</v>
+        <v>1.393517170347966</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6233</v>
+        <v>6236</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>旺玖</t>
+          <t>中湛</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>231.9219005558428</v>
+        <v>232.1255164811716</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>21.5</v>
+        <v>0</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G99" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>46.14035195615092</v>
+        <v>46.8297117891449</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>24.00068922037356</v>
+        <v>9.667865126411858</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5423056105388239</v>
+        <v>0</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,48 +5711,48 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.3016596928865098</v>
+        <v>0.4029301965684577</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6281</v>
+        <v>6233</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>全國電</t>
+          <t>旺玖</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>225.0036341134334</v>
+        <v>231.9219005558428</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>51.5</v>
+        <v>21.5</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G100" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>48.61713906562977</v>
+        <v>46.14035195615092</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>15.51562724375962</v>
+        <v>24.00068922037356</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.521323172512264</v>
+        <v>0.5423056105388239</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.02545849082681</v>
+        <v>0.3016596928865098</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6412</v>
+        <v>6281</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>全國電</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>222.257432625376</v>
+        <v>225.0036341134334</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>78.7</v>
+        <v>51.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.09694487406608</v>
+        <v>48.61713906562977</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>28.53986079364707</v>
+        <v>15.51562724375962</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.3492821225902787</v>
+        <v>0.521323172512264</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.505819703174204</v>
+        <v>-0.02545849082681</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6189</v>
+        <v>6412</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>豐藝</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>221.3273772087615</v>
+        <v>222.257432625376</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>48.4</v>
+        <v>78.7</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>46.92933752020699</v>
+        <v>42.09694487406608</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>9.825229889589249</v>
+        <v>28.53986079364707</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.8825538428144112</v>
+        <v>0.3492821225902787</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.2544643699929629</v>
+        <v>0.505819703174204</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6465</v>
+        <v>6189</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>威潤</t>
+          <t>豐藝</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>215.9219327895048</v>
+        <v>221.3273772087615</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>46.35</v>
+        <v>48.4</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>34.30302225335289</v>
+        <v>46.92933752020699</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>14.94567949304332</v>
+        <v>9.825229889589249</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5984979523824701</v>
+        <v>0.8825538428144112</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.2576580468797793</v>
+        <v>0.2544643699929629</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6216</v>
+        <v>6465</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>威潤</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>215.2316628189612</v>
+        <v>215.9219327895048</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>22.35</v>
+        <v>46.35</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>52.05397440654585</v>
+        <v>34.30302225335289</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>13.85499637527368</v>
+        <v>14.94567949304332</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.4002673443742702</v>
+        <v>0.5984979523824701</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.1025078474719903</v>
+        <v>0.2576580468797793</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6438</v>
+        <v>6216</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>210.4989368543088</v>
+        <v>215.2316628189612</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>147.5</v>
+        <v>22.35</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.17231980711514</v>
+        <v>52.05397440654585</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>17.31674783631032</v>
+        <v>13.85499637527368</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.8245600680753058</v>
+        <v>0.4002673443742702</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>1.250640433700167</v>
+        <v>0.1025078474719903</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6184</v>
+        <v>6438</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>大豐電</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>208.6777790877836</v>
+        <v>210.4989368543088</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>42.1</v>
+        <v>147.5</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>34.32906398888053</v>
+        <v>51.17231980711514</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>14.87520237557796</v>
+        <v>17.31674783631032</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.342687238504321</v>
+        <v>0.8245600680753058</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,48 +6082,48 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0620910981070597</v>
+        <v>1.250640433700167</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6194</v>
+        <v>6184</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>育富</t>
+          <t>大豐電</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>198.5283389064182</v>
+        <v>208.6777790877836</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>29.7</v>
+        <v>42.1</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G107" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>38.96902224474779</v>
+        <v>34.32906398888053</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>26.76549462477533</v>
+        <v>14.87520237557796</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.201592941899357</v>
+        <v>1.342687238504321</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.1147485541792172</v>
+        <v>0.0620910981070597</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6203</v>
+        <v>6194</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>海韻電</t>
+          <t>育富</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>174.3807543751257</v>
+        <v>198.5283389064182</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>60.1</v>
+        <v>29.7</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>30.10696902821288</v>
+        <v>38.96902224474779</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>16.44719003029022</v>
+        <v>26.76549462477533</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1.45793624524921</v>
+        <v>1.201592941899357</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.2224108227605059</v>
+        <v>0.1147485541792172</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6246</v>
+        <v>6203</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>臺龍</t>
+          <t>海韻電</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>165.2662896748806</v>
+        <v>174.3807543751257</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>12.5</v>
+        <v>60.1</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>41.66894239549784</v>
+        <v>30.10696902821288</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>22.95490489518573</v>
+        <v>16.44719003029022</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.6454534796511114</v>
+        <v>1.45793624524921</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.1238699326141078</v>
+        <v>-0.2224108227605059</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6228</v>
+        <v>6246</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>全譜</t>
+          <t>臺龍</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>147.0803998774308</v>
+        <v>165.2662896748806</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>17.65</v>
+        <v>12.5</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>51.44231570794269</v>
+        <v>41.66894239549784</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>9.922472313586788</v>
+        <v>22.95490489518573</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.2309628842644987</v>
+        <v>0.6454534796511114</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0845526163124639</v>
+        <v>0.1238699326141078</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6185</v>
+        <v>6228</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>幃翔</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>136.9822407414973</v>
+        <v>147.0803998774308</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>13.7</v>
+        <v>17.65</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>43.60513601550291</v>
+        <v>51.44231570794269</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.11447799608678</v>
+        <v>9.922472313586788</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.9079645997627586</v>
+        <v>0.2309628842644987</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,48 +6347,48 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0067476912488039</v>
+        <v>-0.0845526163124639</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6235</v>
+        <v>6185</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>華孚</t>
+          <t>幃翔</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>122.0331295033983</v>
+        <v>136.9822407414973</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>39</v>
+        <v>13.7</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G112" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>48.02370380198044</v>
+        <v>43.60513601550291</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>11.59344052740416</v>
+        <v>11.11447799608678</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.4753008388473679</v>
+        <v>0.9079645997627586</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.2291003391023831</v>
+        <v>-0.0067476912488039</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,52 +6410,105 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
+        <v>6235</v>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>華孚</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>122.0331295033983</v>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>48.02370380198044</v>
+      </c>
+      <c r="I113" s="2" t="n">
+        <v>11.59344052740416</v>
+      </c>
+      <c r="J113" s="2" t="n">
+        <v>0.4753008388473679</v>
+      </c>
+      <c r="K113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N113" s="2" t="n">
+        <v>0.2291003391023831</v>
+      </c>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
         <v>6222</v>
       </c>
-      <c r="B113" s="2" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>立軒</t>
         </is>
       </c>
-      <c r="C113" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D113" s="2" t="n">
+      <c r="C114" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D114" s="2" t="n">
         <v>55.58098052647912</v>
       </c>
-      <c r="E113" s="2" t="n">
+      <c r="E114" s="2" t="n">
         <v>20.1</v>
       </c>
-      <c r="F113" s="2" t="inlineStr">
+      <c r="F114" s="2" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="G113" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H113" s="2" t="n">
+      <c r="G114" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H114" s="2" t="n">
         <v>50.8063582316648</v>
       </c>
-      <c r="I113" s="2" t="n">
+      <c r="I114" s="2" t="n">
         <v>12.27172778168297</v>
       </c>
-      <c r="J113" s="2" t="n">
+      <c r="J114" s="2" t="n">
         <v>0.4829914558811455</v>
       </c>
-      <c r="K113" s="2" t="n">
+      <c r="K114" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M113" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N113" s="2" t="n">
+      <c r="L114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N114" s="2" t="n">
         <v>0.2648787358799002</v>
       </c>
-      <c r="O113" s="2" t="inlineStr">
+      <c r="O114" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>